<commit_message>
apply plot improvements to best_TM17_20260728 results
</commit_message>
<xml_diff>
--- a/utilities/trucks/trucks_2026_update/models/evaluation/best_TM17_20260728/truck_model_evaluation.xlsx
+++ b/utilities/trucks/trucks_2026_update/models/evaluation/best_TM17_20260728/truck_model_evaluation.xlsx
@@ -15,7 +15,6 @@
     <sheet name="Total Truck VMT" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Trip Distributions Plots" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Scatter Plots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="VMT Comparison" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -524,61 +523,6 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5715000" cy="3810000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>28</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5715000" cy="3810000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -895,7 +839,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28 21:47</t>
+          <t>2026-08-04 15:21</t>
         </is>
       </c>
     </row>
@@ -2393,33 +2337,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Heavy Trucks (HV)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Very Small, Small &amp; Medium Trucks (SM)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
rename validation_table.shp to assinged_volumnes for old experiments
</commit_message>
<xml_diff>
--- a/utilities/trucks/trucks_2026_update/models/evaluation/best_TM17_20260728/truck_model_evaluation.xlsx
+++ b/utilities/trucks/trucks_2026_update/models/evaluation/best_TM17_20260728/truck_model_evaluation.xlsx
@@ -2337,4 +2337,225 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007853A55483E9744FB060D23556A13F64" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a83bcbbd6d554c58145aac23e8d59d9f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eb8c3add-cb83-4098-bf9b-bebb1bb4c1ed" xmlns:ns3="87dae7b4-e272-45c2-8afb-ad5981533a8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5cc5c4ee65facea36e7fe995ddcc67a1" ns2:_="" ns3:_="">
+    <xsd:import namespace="eb8c3add-cb83-4098-bf9b-bebb1bb4c1ed"/>
+    <xsd:import namespace="87dae7b4-e272-45c2-8afb-ad5981533a8e"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="eb8c3add-cb83-4098-bf9b-bebb1bb4c1ed" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="b5d298e1-810f-4711-8be9-ef4702f2a38a" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="87dae7b4-e272-45c2-8afb-ad5981533a8e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{304ecca4-c6f5-4a6b-87b7-c47348f4eacc}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="87dae7b4-e272-45c2-8afb-ad5981533a8e">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="87dae7b4-e272-45c2-8afb-ad5981533a8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb8c3add-cb83-4098-bf9b-bebb1bb4c1ed">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51601D02-7F99-41EF-8541-E4CE085BC1D1}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AF63513C-3E40-47F9-AE07-6383D0C17A0C}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0253B9C1-3EFF-42CC-AA1C-E2A298E57FD3}"/>
 </file>
</xml_diff>